<commit_message>
Align profiles with workbook labels, NA handling, blueprint verification
- Country profiles: Excel-accurate INDEX_BLUEPRINT, DATA NOT AVAILABLE for gaps
- Loader: workbookVariableUnavailable; ingest/validate script updates
- Indicators page: matching pillar and block names; verify:data npm script
- Regenerated ingested data from Part 3 workbook

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/the index/part 3 democracy.xlsx
+++ b/the index/part 3 democracy.xlsx
@@ -14,17 +14,17 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={1d3fd798-2daf-4bba-92e0-8dc8db665a28}</author>
-    <author>tc={29a1af87-1346-463f-8f03-b9effe2c8c91}</author>
-    <author>tc={41de4c90-42f5-4b59-9a23-f476b638c110}</author>
-    <author>tc={6ae99fcb-8d84-4964-a257-79aa41324616}</author>
-    <author>tc={7b505acc-a69e-4e9e-a2ab-478b64f70be2}</author>
-    <author>tc={890297cc-649d-4427-ba0f-c61a539b3fce}</author>
-    <author>tc={94e1fcfa-c9ea-43d0-8436-bbe0f25179a6}</author>
-    <author>tc={9508b233-b384-475a-bc85-cfb9deb6fc86}</author>
+    <author>tc={0dd53e57-e4eb-4ce2-a6e4-2fffe9bd9510}</author>
+    <author>tc={1832685e-04d8-4fd6-9fdd-0b6a3e125c27}</author>
+    <author>tc={3c68618e-dab6-4486-a721-101acbe1a00c}</author>
+    <author>tc={5351f367-8777-4ac1-8886-ea740ea8190d}</author>
+    <author>tc={5840afd9-6059-4d30-9a4e-7b00527affe3}</author>
+    <author>tc={df0fc6e2-ee0f-4daa-a3d9-08113dbe6556}</author>
+    <author>tc={e6037a84-b7cd-4e81-91d9-cea8c728bbe7}</author>
+    <author>tc={ea62b956-8511-42c5-94f6-b7e302d2143a}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{1d3fd798-2daf-4bba-92e0-8dc8db665a28}" ref="I241">
+    <comment authorId="0" xr:uid="{0dd53e57-e4eb-4ce2-a6e4-2fffe9bd9510}" ref="I241">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -33,7 +33,52 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{29a1af87-1346-463f-8f03-b9effe2c8c91}" ref="I258">
+    <comment authorId="1" xr:uid="{1832685e-04d8-4fd6-9fdd-0b6a3e125c27}" ref="I358">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	n/a
+</t>
+      </text>
+    </comment>
+    <comment authorId="2" xr:uid="{3c68618e-dab6-4486-a721-101acbe1a00c}" ref="A1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	n/a
+</t>
+      </text>
+    </comment>
+    <comment authorId="3" xr:uid="{5351f367-8777-4ac1-8886-ea740ea8190d}" ref="I457">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	n/a
+</t>
+      </text>
+    </comment>
+    <comment authorId="4" xr:uid="{5840afd9-6059-4d30-9a4e-7b00527affe3}" ref="I102">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	no hi ha info al WB
+</t>
+      </text>
+    </comment>
+    <comment authorId="5" xr:uid="{df0fc6e2-ee0f-4daa-a3d9-08113dbe6556}" ref="I262">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	n/a
+</t>
+      </text>
+    </comment>
+    <comment authorId="6" xr:uid="{e6037a84-b7cd-4e81-91d9-cea8c728bbe7}" ref="I258">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -42,52 +87,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{41de4c90-42f5-4b59-9a23-f476b638c110}" ref="A1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	n/a
-</t>
-      </text>
-    </comment>
-    <comment authorId="3" xr:uid="{6ae99fcb-8d84-4964-a257-79aa41324616}" ref="I358">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	n/a
-</t>
-      </text>
-    </comment>
-    <comment authorId="4" xr:uid="{7b505acc-a69e-4e9e-a2ab-478b64f70be2}" ref="I262">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	n/a
-</t>
-      </text>
-    </comment>
-    <comment authorId="5" xr:uid="{890297cc-649d-4427-ba0f-c61a539b3fce}" ref="I102">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	no hi ha info al WB
-</t>
-      </text>
-    </comment>
-    <comment authorId="6" xr:uid="{94e1fcfa-c9ea-43d0-8436-bbe0f25179a6}" ref="I379">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	n/a
-</t>
-      </text>
-    </comment>
-    <comment authorId="7" xr:uid="{9508b233-b384-475a-bc85-cfb9deb6fc86}" ref="I457">
+    <comment authorId="7" xr:uid="{ea62b956-8511-42c5-94f6-b7e302d2143a}" ref="I379">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -103,21 +103,21 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={2d155f64-6a41-46a8-93d8-7ed7cc5bcb63}</author>
-    <author>tc={34cf2329-75ad-4453-9ae9-d64cbd05383e}</author>
-    <author>tc={49cea25f-b8a7-4565-8e78-8a1b55a1835a}</author>
-    <author>tc={4bf6b79e-8e8b-4959-a3a7-6d94f3eb378d}</author>
-    <author>tc={51fb298c-3e16-4bea-8701-803f392ab6fb}</author>
-    <author>tc={5798692c-0381-405f-9f72-56d1f62cd02f}</author>
-    <author>tc={5d8f961c-71b2-41f5-8d61-4fdc80e2960a}</author>
-    <author>tc={678329c5-5603-484b-b813-831252ddfc47}</author>
-    <author>tc={86d31ca3-41ac-4c56-93be-c209c86d1183}</author>
-    <author>tc={885884d4-3445-475f-a57e-dbb53ca66352}</author>
-    <author>tc={945838cc-33b8-4b02-a561-ed5402883a35}</author>
-    <author>tc={d5eeed0e-7c80-4710-a51a-468e03b26e59}</author>
+    <author>tc={1c617a85-4c98-477a-b470-d2c7b41fd803}</author>
+    <author>tc={21004543-e884-4f77-a3e1-a61cede9b0cc}</author>
+    <author>tc={319b39de-6797-4a92-bb6d-4a72cd126bd3}</author>
+    <author>tc={37bab43c-7ff1-44b8-a17f-59cb8fe7cd70}</author>
+    <author>tc={402856c9-3508-4207-9010-512102695bc7}</author>
+    <author>tc={583daa39-7e7c-4875-9e8f-545cb43d8101}</author>
+    <author>tc={629fe1e2-e12b-46a5-bf71-31cb181d8216}</author>
+    <author>tc={82d6ed77-6868-4e7b-ac28-f14733b1ea09}</author>
+    <author>tc={8ad5a8b8-4025-40e6-a5a6-20a0eaf51c92}</author>
+    <author>tc={a587d043-59b2-4fb9-9bfb-6a42272ac387}</author>
+    <author>tc={e49e8ad0-0dea-486e-8923-edb454bd3887}</author>
+    <author>tc={f7c4dd04-746b-4d8d-9dd3-c0b20adce83e}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{2d155f64-6a41-46a8-93d8-7ed7cc5bcb63}" ref="I65">
+    <comment authorId="0" xr:uid="{1c617a85-4c98-477a-b470-d2c7b41fd803}" ref="I141">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -126,7 +126,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{34cf2329-75ad-4453-9ae9-d64cbd05383e}" ref="I331">
+    <comment authorId="1" xr:uid="{21004543-e884-4f77-a3e1-a61cede9b0cc}" ref="I331">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -135,7 +135,16 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{49cea25f-b8a7-4565-8e78-8a1b55a1835a}" ref="I217">
+    <comment authorId="2" xr:uid="{319b39de-6797-4a92-bb6d-4a72cd126bd3}" ref="I222">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	not available
+</t>
+      </text>
+    </comment>
+    <comment authorId="3" xr:uid="{37bab43c-7ff1-44b8-a17f-59cb8fe7cd70}" ref="I224">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -144,25 +153,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="3" xr:uid="{4bf6b79e-8e8b-4959-a3a7-6d94f3eb378d}" ref="I222">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	not available
-</t>
-      </text>
-    </comment>
-    <comment authorId="4" xr:uid="{51fb298c-3e16-4bea-8701-803f392ab6fb}" ref="I223">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	notavailable
-</t>
-      </text>
-    </comment>
-    <comment authorId="5" xr:uid="{5798692c-0381-405f-9f72-56d1f62cd02f}" ref="I179">
+    <comment authorId="4" xr:uid="{402856c9-3508-4207-9010-512102695bc7}" ref="I61">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -171,7 +162,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="6" xr:uid="{5d8f961c-71b2-41f5-8d61-4fdc80e2960a}" ref="I49">
+    <comment authorId="5" xr:uid="{583daa39-7e7c-4875-9e8f-545cb43d8101}" ref="I65">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -180,7 +171,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="7" xr:uid="{678329c5-5603-484b-b813-831252ddfc47}" ref="I61">
+    <comment authorId="6" xr:uid="{629fe1e2-e12b-46a5-bf71-31cb181d8216}" ref="I219">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -189,7 +180,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="8" xr:uid="{86d31ca3-41ac-4c56-93be-c209c86d1183}" ref="I141">
+    <comment authorId="7" xr:uid="{82d6ed77-6868-4e7b-ac28-f14733b1ea09}" ref="I59">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -198,7 +189,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="9" xr:uid="{885884d4-3445-475f-a57e-dbb53ca66352}" ref="I219">
+    <comment authorId="8" xr:uid="{8ad5a8b8-4025-40e6-a5a6-20a0eaf51c92}" ref="I217">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -207,7 +198,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="10" xr:uid="{945838cc-33b8-4b02-a561-ed5402883a35}" ref="I59">
+    <comment authorId="9" xr:uid="{a587d043-59b2-4fb9-9bfb-6a42272ac387}" ref="I49">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -216,12 +207,21 @@
 </t>
       </text>
     </comment>
-    <comment authorId="11" xr:uid="{d5eeed0e-7c80-4710-a51a-468e03b26e59}" ref="I224">
+    <comment authorId="10" xr:uid="{e49e8ad0-0dea-486e-8923-edb454bd3887}" ref="I179">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
 	n/a
+</t>
+      </text>
+    </comment>
+    <comment authorId="11" xr:uid="{f7c4dd04-746b-4d8d-9dd3-c0b20adce83e}" ref="I223">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	notavailable
 </t>
       </text>
     </comment>
@@ -917,6 +917,554 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'SOUTH AMERICA'!$K$1</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'SOUTH AMERICA'!$A$2:$A$1061</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'SOUTH AMERICA'!$K$2:$K$1061</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'SOUTH AMERICA'!$A$1</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'SOUTH AMERICA'!$A$2:$A$1061</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'SOUTH AMERICA'!$A$2:$A$1061</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1220275267"/>
+        <c:axId val="1333601652"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1220275267"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:spPr/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1333601652"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1333601652"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1220275267"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>CENTROAMERICA!$K$1</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>CENTROAMERICA!$A$2:$A$962</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>CENTROAMERICA!$K$2:$K$962</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>CENTROAMERICA!$A$1</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>CENTROAMERICA!$A$2:$A$962</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>CENTROAMERICA!$A$2:$A$962</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1233030467"/>
+        <c:axId val="1950501557"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1233030467"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:spPr/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1950501557"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1950501557"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1233030467"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>CENTROAMERICA!$O$20</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1969812328"/>
+        <c:axId val="1569116844"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1969812328"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:spPr/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1569116844"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1569116844"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:crossAx val="1969812328"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
 <file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
 <Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
 </file>
@@ -926,17 +1474,94 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>904875</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5715000" cy="3533775"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 1" title="Gràfic"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>771525</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5715000" cy="3533775"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 2" title="Gràfic"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5715000" cy="3533775"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 3" title="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Ariadna Bertran i Celaya" id="{430bbbab-8eb6-402a-bec7-ae249609f4d5}" providerId="google-sheets"/>
-  <x18tc:person displayName="Roser" id="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" providerId="google-sheets"/>
+  <x18tc:person displayName="Ariadna Bertran i Celaya" id="{c47a4ff3-eb60-4f69-bccc-eb5bc4d08067}" providerId="google-sheets"/>
+  <x18tc:person displayName="Roser" id="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1136,28 +1761,28 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="I258" dT="2026-04-18T19:17:24.00" personId="{430bbbab-8eb6-402a-bec7-ae249609f4d5}" id="{29a1af87-1346-463f-8f03-b9effe2c8c91}" done="1">
+  <x18tc:threadedComment ref="I258" dT="2026-04-18T19:17:24.00" personId="{c47a4ff3-eb60-4f69-bccc-eb5bc4d08067}" id="{e6037a84-b7cd-4e81-91d9-cea8c728bbe7}" done="1">
     <x18tc:text xml:space="preserve">no hi ha dades al WB</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I262" dT="2026-04-18T20:43:48.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{7b505acc-a69e-4e9e-a2ab-478b64f70be2}" done="1">
+  <x18tc:threadedComment ref="I262" dT="2026-04-18T20:43:48.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{df0fc6e2-ee0f-4daa-a3d9-08113dbe6556}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I379" dT="2026-04-18T20:44:28.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{94e1fcfa-c9ea-43d0-8436-bbe0f25179a6}" done="1">
+  <x18tc:threadedComment ref="I379" dT="2026-04-18T20:44:28.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{ea62b956-8511-42c5-94f6-b7e302d2143a}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I358" dT="2026-04-19T13:51:11.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{6ae99fcb-8d84-4964-a257-79aa41324616}" done="1">
+  <x18tc:threadedComment ref="I358" dT="2026-04-19T13:51:11.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{1832685e-04d8-4fd6-9fdd-0b6a3e125c27}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I457" dT="2026-04-18T20:44:49.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{9508b233-b384-475a-bc85-cfb9deb6fc86}" done="1">
+  <x18tc:threadedComment ref="I457" dT="2026-04-18T20:44:49.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{5351f367-8777-4ac1-8886-ea740ea8190d}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I241" dT="2026-04-19T13:50:08.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{1d3fd798-2daf-4bba-92e0-8dc8db665a28}" done="1">
+  <x18tc:threadedComment ref="I241" dT="2026-04-19T13:50:08.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{0dd53e57-e4eb-4ce2-a6e4-2fffe9bd9510}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-04-19T13:50:44.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{41de4c90-42f5-4b59-9a23-f476b638c110}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-04-19T13:50:44.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{3c68618e-dab6-4486-a721-101acbe1a00c}" done="0">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I102" dT="2026-04-18T19:14:13.00" personId="{430bbbab-8eb6-402a-bec7-ae249609f4d5}" id="{890297cc-649d-4427-ba0f-c61a539b3fce}" done="1">
+  <x18tc:threadedComment ref="I102" dT="2026-04-18T19:14:13.00" personId="{c47a4ff3-eb60-4f69-bccc-eb5bc4d08067}" id="{5840afd9-6059-4d30-9a4e-7b00527affe3}" done="1">
     <x18tc:text xml:space="preserve">no hi ha info al WB</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1165,40 +1790,40 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="I65" dT="2026-04-19T14:01:38.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{2d155f64-6a41-46a8-93d8-7ed7cc5bcb63}" done="1">
+  <x18tc:threadedComment ref="I65" dT="2026-04-19T14:01:38.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{583daa39-7e7c-4875-9e8f-545cb43d8101}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I217" dT="2026-04-19T14:01:10.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{49cea25f-b8a7-4565-8e78-8a1b55a1835a}" done="1">
+  <x18tc:threadedComment ref="I217" dT="2026-04-19T14:01:10.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{8ad5a8b8-4025-40e6-a5a6-20a0eaf51c92}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I222" dT="2026-04-19T12:32:03.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{4bf6b79e-8e8b-4959-a3a7-6d94f3eb378d}" done="1">
+  <x18tc:threadedComment ref="I222" dT="2026-04-19T12:32:03.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{319b39de-6797-4a92-bb6d-4a72cd126bd3}" done="1">
     <x18tc:text xml:space="preserve">not available</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I179" dT="2026-04-19T14:01:04.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{5798692c-0381-405f-9f72-56d1f62cd02f}" done="1">
+  <x18tc:threadedComment ref="I179" dT="2026-04-19T14:01:04.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{e49e8ad0-0dea-486e-8923-edb454bd3887}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I219" dT="2026-04-19T12:32:09.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{885884d4-3445-475f-a57e-dbb53ca66352}" done="1">
+  <x18tc:threadedComment ref="I219" dT="2026-04-19T12:32:09.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{629fe1e2-e12b-46a5-bf71-31cb181d8216}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I141" dT="2026-04-19T14:00:55.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{86d31ca3-41ac-4c56-93be-c209c86d1183}" done="1">
+  <x18tc:threadedComment ref="I141" dT="2026-04-19T14:00:55.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{1c617a85-4c98-477a-b470-d2c7b41fd803}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I61" dT="2026-04-19T15:10:14.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{678329c5-5603-484b-b813-831252ddfc47}" done="1">
+  <x18tc:threadedComment ref="I61" dT="2026-04-19T15:10:14.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{402856c9-3508-4207-9010-512102695bc7}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I223" dT="2026-04-19T12:34:30.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{51fb298c-3e16-4bea-8701-803f392ab6fb}" done="1">
+  <x18tc:threadedComment ref="I223" dT="2026-04-19T12:34:30.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{f7c4dd04-746b-4d8d-9dd3-c0b20adce83e}" done="1">
     <x18tc:text xml:space="preserve">notavailable</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I331" dT="2026-04-19T14:00:16.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{34cf2329-75ad-4453-9ae9-d64cbd05383e}" done="1">
+  <x18tc:threadedComment ref="I331" dT="2026-04-19T14:00:16.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{21004543-e884-4f77-a3e1-a61cede9b0cc}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I59" dT="2026-04-19T15:01:09.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{945838cc-33b8-4b02-a561-ed5402883a35}" done="1">
+  <x18tc:threadedComment ref="I59" dT="2026-04-19T15:01:09.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{82d6ed77-6868-4e7b-ac28-f14733b1ea09}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I224" dT="2026-04-19T12:36:54.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{d5eeed0e-7c80-4710-a51a-468e03b26e59}" done="1">
+  <x18tc:threadedComment ref="I224" dT="2026-04-19T12:36:54.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{37bab43c-7ff1-44b8-a17f-59cb8fe7cd70}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I49" dT="2026-04-19T14:25:22.00" personId="{d6b8369a-e8e7-40e2-9c61-3ea2d32efefe}" id="{5d8f961c-71b2-41f5-8d61-4fdc80e2960a}" done="1">
+  <x18tc:threadedComment ref="I49" dT="2026-04-19T14:25:22.00" personId="{d57fe9fb-c744-4322-9c8e-9f25704e3457}" id="{a587d043-59b2-4fb9-9bfb-6a42272ac387}" done="1">
     <x18tc:text xml:space="preserve">n/a</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -14899,20 +15524,40 @@
     <mergeCell ref="G192:G193"/>
     <mergeCell ref="F194:F195"/>
     <mergeCell ref="G194:G195"/>
+    <mergeCell ref="B259:B262"/>
+    <mergeCell ref="C259:C262"/>
+    <mergeCell ref="B263:B269"/>
+    <mergeCell ref="C263:C269"/>
+    <mergeCell ref="B270:B273"/>
+    <mergeCell ref="C270:C273"/>
+    <mergeCell ref="C276:C286"/>
+    <mergeCell ref="B192:B195"/>
+    <mergeCell ref="C192:C195"/>
+    <mergeCell ref="A198:A234"/>
+    <mergeCell ref="B198:B208"/>
+    <mergeCell ref="C198:C208"/>
+    <mergeCell ref="C209:C219"/>
+    <mergeCell ref="A237:A273"/>
+    <mergeCell ref="C326:C336"/>
+    <mergeCell ref="D326:D336"/>
     <mergeCell ref="B337:B340"/>
-    <mergeCell ref="B348:B351"/>
-    <mergeCell ref="A276:A312"/>
-    <mergeCell ref="B276:B286"/>
-    <mergeCell ref="A315:A351"/>
-    <mergeCell ref="B315:B325"/>
-    <mergeCell ref="C315:C325"/>
-    <mergeCell ref="D315:D325"/>
+    <mergeCell ref="C337:C340"/>
+    <mergeCell ref="C341:C347"/>
     <mergeCell ref="D341:D347"/>
+    <mergeCell ref="E276:E279"/>
+    <mergeCell ref="E280:E281"/>
+    <mergeCell ref="E315:E318"/>
+    <mergeCell ref="E321:E323"/>
+    <mergeCell ref="E324:E325"/>
+    <mergeCell ref="E326:E329"/>
+    <mergeCell ref="E330:E333"/>
+    <mergeCell ref="E334:E336"/>
+    <mergeCell ref="E337:E338"/>
+    <mergeCell ref="E339:E340"/>
+    <mergeCell ref="E341:E344"/>
     <mergeCell ref="E345:E347"/>
     <mergeCell ref="E348:E349"/>
     <mergeCell ref="E350:E351"/>
-    <mergeCell ref="E354:E357"/>
-    <mergeCell ref="E358:E359"/>
     <mergeCell ref="E360:E362"/>
     <mergeCell ref="E363:E364"/>
     <mergeCell ref="E365:E368"/>
@@ -14936,20 +15581,20 @@
     <mergeCell ref="E419:E422"/>
     <mergeCell ref="E423:E425"/>
     <mergeCell ref="E426:E427"/>
+    <mergeCell ref="E428:E429"/>
+    <mergeCell ref="E432:E435"/>
+    <mergeCell ref="E436:E437"/>
+    <mergeCell ref="E438:E440"/>
+    <mergeCell ref="E441:E442"/>
+    <mergeCell ref="E465:E466"/>
+    <mergeCell ref="E467:E468"/>
+    <mergeCell ref="E443:E446"/>
+    <mergeCell ref="E447:E450"/>
     <mergeCell ref="E451:E453"/>
     <mergeCell ref="E454:E455"/>
     <mergeCell ref="E456:E457"/>
     <mergeCell ref="E458:E461"/>
     <mergeCell ref="E462:E464"/>
-    <mergeCell ref="E465:E466"/>
-    <mergeCell ref="E467:E468"/>
-    <mergeCell ref="E428:E429"/>
-    <mergeCell ref="E432:E435"/>
-    <mergeCell ref="E436:E437"/>
-    <mergeCell ref="E438:E440"/>
-    <mergeCell ref="E441:E442"/>
-    <mergeCell ref="E443:E446"/>
-    <mergeCell ref="E447:E450"/>
     <mergeCell ref="B170:B180"/>
     <mergeCell ref="C170:C180"/>
     <mergeCell ref="D181:D184"/>
@@ -14969,81 +15614,68 @@
     <mergeCell ref="D159:D169"/>
     <mergeCell ref="D270:D273"/>
     <mergeCell ref="D276:D286"/>
-    <mergeCell ref="E276:E279"/>
-    <mergeCell ref="E280:E281"/>
-    <mergeCell ref="E315:E318"/>
-    <mergeCell ref="E334:E336"/>
-    <mergeCell ref="E337:E338"/>
-    <mergeCell ref="E339:E340"/>
-    <mergeCell ref="E341:E344"/>
+    <mergeCell ref="E354:E357"/>
+    <mergeCell ref="E358:E359"/>
+    <mergeCell ref="C432:C442"/>
+    <mergeCell ref="D432:D442"/>
+    <mergeCell ref="B419:B425"/>
+    <mergeCell ref="C419:C425"/>
+    <mergeCell ref="D419:D425"/>
+    <mergeCell ref="B426:B429"/>
+    <mergeCell ref="C426:C429"/>
+    <mergeCell ref="D426:D429"/>
+    <mergeCell ref="B432:B442"/>
+    <mergeCell ref="C458:C464"/>
+    <mergeCell ref="D458:D464"/>
+    <mergeCell ref="B443:B453"/>
+    <mergeCell ref="C443:C453"/>
+    <mergeCell ref="D443:D453"/>
+    <mergeCell ref="B454:B457"/>
+    <mergeCell ref="C454:C457"/>
+    <mergeCell ref="D454:D457"/>
+    <mergeCell ref="B458:B464"/>
+    <mergeCell ref="A276:A312"/>
+    <mergeCell ref="B276:B286"/>
+    <mergeCell ref="A315:A351"/>
+    <mergeCell ref="B315:B325"/>
+    <mergeCell ref="C315:C325"/>
+    <mergeCell ref="D315:D325"/>
+    <mergeCell ref="D337:D340"/>
+    <mergeCell ref="D348:D351"/>
+    <mergeCell ref="C376:C379"/>
+    <mergeCell ref="C380:C386"/>
+    <mergeCell ref="D380:D386"/>
+    <mergeCell ref="C387:C390"/>
+    <mergeCell ref="D387:D390"/>
     <mergeCell ref="C393:C403"/>
+    <mergeCell ref="D393:D403"/>
+    <mergeCell ref="B348:B351"/>
+    <mergeCell ref="C348:C351"/>
+    <mergeCell ref="C354:C364"/>
+    <mergeCell ref="D354:D364"/>
+    <mergeCell ref="C365:C375"/>
+    <mergeCell ref="D365:D375"/>
+    <mergeCell ref="D376:D379"/>
+    <mergeCell ref="A354:A390"/>
+    <mergeCell ref="A393:A429"/>
+    <mergeCell ref="A432:A468"/>
+    <mergeCell ref="B326:B336"/>
+    <mergeCell ref="B341:B347"/>
+    <mergeCell ref="B354:B364"/>
+    <mergeCell ref="B365:B375"/>
+    <mergeCell ref="B376:B379"/>
+    <mergeCell ref="B380:B386"/>
+    <mergeCell ref="B387:B390"/>
+    <mergeCell ref="B393:B403"/>
     <mergeCell ref="B404:B414"/>
     <mergeCell ref="C404:C414"/>
-    <mergeCell ref="B341:B347"/>
-    <mergeCell ref="C341:C347"/>
-    <mergeCell ref="A354:A390"/>
-    <mergeCell ref="B354:B364"/>
-    <mergeCell ref="C354:C364"/>
-    <mergeCell ref="C365:C375"/>
-    <mergeCell ref="A393:A429"/>
-    <mergeCell ref="B380:B386"/>
-    <mergeCell ref="C380:C386"/>
-    <mergeCell ref="B387:B390"/>
-    <mergeCell ref="C387:C390"/>
-    <mergeCell ref="B365:B375"/>
-    <mergeCell ref="B393:B403"/>
+    <mergeCell ref="D404:D414"/>
     <mergeCell ref="B415:B418"/>
     <mergeCell ref="C415:C418"/>
-    <mergeCell ref="B419:B425"/>
-    <mergeCell ref="C419:C425"/>
-    <mergeCell ref="B426:B429"/>
-    <mergeCell ref="C426:C429"/>
-    <mergeCell ref="C432:C442"/>
-    <mergeCell ref="C443:C453"/>
-    <mergeCell ref="C454:C457"/>
-    <mergeCell ref="C458:C464"/>
+    <mergeCell ref="D415:D418"/>
+    <mergeCell ref="B465:B468"/>
     <mergeCell ref="C465:C468"/>
-    <mergeCell ref="B432:B442"/>
-    <mergeCell ref="B443:B453"/>
-    <mergeCell ref="B454:B457"/>
-    <mergeCell ref="B458:B464"/>
-    <mergeCell ref="B465:B468"/>
-    <mergeCell ref="D443:D453"/>
-    <mergeCell ref="A432:A468"/>
-    <mergeCell ref="D415:D418"/>
-    <mergeCell ref="D419:D425"/>
-    <mergeCell ref="D426:D429"/>
-    <mergeCell ref="D432:D442"/>
-    <mergeCell ref="D454:D457"/>
-    <mergeCell ref="D458:D464"/>
     <mergeCell ref="D465:D468"/>
-    <mergeCell ref="B259:B262"/>
-    <mergeCell ref="C259:C262"/>
-    <mergeCell ref="B263:B269"/>
-    <mergeCell ref="C263:C269"/>
-    <mergeCell ref="B270:B273"/>
-    <mergeCell ref="C270:C273"/>
-    <mergeCell ref="C276:C286"/>
-    <mergeCell ref="B192:B195"/>
-    <mergeCell ref="C192:C195"/>
-    <mergeCell ref="A198:A234"/>
-    <mergeCell ref="B198:B208"/>
-    <mergeCell ref="C198:C208"/>
-    <mergeCell ref="C209:C219"/>
-    <mergeCell ref="A237:A273"/>
-    <mergeCell ref="C337:C340"/>
-    <mergeCell ref="D337:D340"/>
-    <mergeCell ref="C348:C351"/>
-    <mergeCell ref="D348:D351"/>
-    <mergeCell ref="D354:D364"/>
-    <mergeCell ref="D365:D375"/>
-    <mergeCell ref="B376:B379"/>
-    <mergeCell ref="C376:C379"/>
-    <mergeCell ref="D376:D379"/>
-    <mergeCell ref="D380:D386"/>
-    <mergeCell ref="D387:D390"/>
-    <mergeCell ref="D393:D403"/>
-    <mergeCell ref="D404:D414"/>
     <mergeCell ref="E139:E141"/>
     <mergeCell ref="B142:B145"/>
     <mergeCell ref="C142:C145"/>
@@ -15155,6 +15787,169 @@
     <mergeCell ref="E267:E269"/>
     <mergeCell ref="E270:E271"/>
     <mergeCell ref="E272:E273"/>
+    <mergeCell ref="F319:F320"/>
+    <mergeCell ref="G319:G320"/>
+    <mergeCell ref="F306:F308"/>
+    <mergeCell ref="F309:F310"/>
+    <mergeCell ref="G309:G310"/>
+    <mergeCell ref="F311:F312"/>
+    <mergeCell ref="G311:G312"/>
+    <mergeCell ref="F315:F318"/>
+    <mergeCell ref="G315:G318"/>
+    <mergeCell ref="H241:H242"/>
+    <mergeCell ref="H332:H333"/>
+    <mergeCell ref="I332:I333"/>
+    <mergeCell ref="J332:J333"/>
+    <mergeCell ref="H215:H216"/>
+    <mergeCell ref="I215:I216"/>
+    <mergeCell ref="K237:K273"/>
+    <mergeCell ref="I241:I242"/>
+    <mergeCell ref="J241:J242"/>
+    <mergeCell ref="K276:K312"/>
+    <mergeCell ref="K315:K351"/>
+    <mergeCell ref="H371:H372"/>
+    <mergeCell ref="H410:H411"/>
+    <mergeCell ref="I410:I411"/>
+    <mergeCell ref="J410:J411"/>
+    <mergeCell ref="H358:H359"/>
+    <mergeCell ref="H449:H450"/>
+    <mergeCell ref="I449:I450"/>
+    <mergeCell ref="J449:J450"/>
+    <mergeCell ref="K354:K390"/>
+    <mergeCell ref="I358:I359"/>
+    <mergeCell ref="J358:J359"/>
+    <mergeCell ref="I371:I372"/>
+    <mergeCell ref="J371:J372"/>
+    <mergeCell ref="K393:K429"/>
+    <mergeCell ref="K432:K468"/>
+    <mergeCell ref="F204:F206"/>
+    <mergeCell ref="G204:G206"/>
+    <mergeCell ref="F209:F212"/>
+    <mergeCell ref="G209:G212"/>
+    <mergeCell ref="F174:F177"/>
+    <mergeCell ref="G174:G177"/>
+    <mergeCell ref="F198:F201"/>
+    <mergeCell ref="G198:G201"/>
+    <mergeCell ref="K198:K234"/>
+    <mergeCell ref="F202:F203"/>
+    <mergeCell ref="G202:G203"/>
+    <mergeCell ref="J215:J216"/>
+    <mergeCell ref="I254:I255"/>
+    <mergeCell ref="J254:J255"/>
+    <mergeCell ref="F280:F281"/>
+    <mergeCell ref="G280:G281"/>
+    <mergeCell ref="F282:F284"/>
+    <mergeCell ref="G282:G284"/>
+    <mergeCell ref="G285:G286"/>
+    <mergeCell ref="H254:H255"/>
+    <mergeCell ref="H293:H294"/>
+    <mergeCell ref="I293:I294"/>
+    <mergeCell ref="J293:J294"/>
+    <mergeCell ref="F300:F301"/>
+    <mergeCell ref="G300:G301"/>
+    <mergeCell ref="F302:F305"/>
+    <mergeCell ref="G302:G305"/>
+    <mergeCell ref="G306:G308"/>
+    <mergeCell ref="G334:G336"/>
+    <mergeCell ref="G337:G338"/>
+    <mergeCell ref="G399:G401"/>
+    <mergeCell ref="G402:G403"/>
+    <mergeCell ref="G378:G379"/>
+    <mergeCell ref="G380:G383"/>
+    <mergeCell ref="G384:G386"/>
+    <mergeCell ref="G387:G388"/>
+    <mergeCell ref="G389:G390"/>
+    <mergeCell ref="G393:G396"/>
+    <mergeCell ref="G397:G398"/>
+    <mergeCell ref="F412:F414"/>
+    <mergeCell ref="G412:G414"/>
+    <mergeCell ref="F415:F416"/>
+    <mergeCell ref="G415:G416"/>
+    <mergeCell ref="F417:F418"/>
+    <mergeCell ref="G417:G418"/>
+    <mergeCell ref="G419:G422"/>
+    <mergeCell ref="F419:F422"/>
+    <mergeCell ref="F423:F425"/>
+    <mergeCell ref="F426:F427"/>
+    <mergeCell ref="F428:F429"/>
+    <mergeCell ref="F432:F435"/>
+    <mergeCell ref="F436:F437"/>
+    <mergeCell ref="F438:F440"/>
+    <mergeCell ref="G423:G425"/>
+    <mergeCell ref="G426:G427"/>
+    <mergeCell ref="G428:G429"/>
+    <mergeCell ref="G432:G435"/>
+    <mergeCell ref="G436:G437"/>
+    <mergeCell ref="G438:G440"/>
+    <mergeCell ref="G441:G442"/>
+    <mergeCell ref="F462:F464"/>
+    <mergeCell ref="F465:F466"/>
+    <mergeCell ref="F467:F468"/>
+    <mergeCell ref="F441:F442"/>
+    <mergeCell ref="F443:F446"/>
+    <mergeCell ref="F447:F450"/>
+    <mergeCell ref="F451:F453"/>
+    <mergeCell ref="F454:F455"/>
+    <mergeCell ref="F456:F457"/>
+    <mergeCell ref="F458:F461"/>
+    <mergeCell ref="G465:G466"/>
+    <mergeCell ref="G467:G468"/>
+    <mergeCell ref="G443:G446"/>
+    <mergeCell ref="G447:G450"/>
+    <mergeCell ref="G451:G453"/>
+    <mergeCell ref="G454:G455"/>
+    <mergeCell ref="G456:G457"/>
+    <mergeCell ref="G458:G461"/>
+    <mergeCell ref="G462:G464"/>
+    <mergeCell ref="F321:F323"/>
+    <mergeCell ref="G321:G323"/>
+    <mergeCell ref="F324:F325"/>
+    <mergeCell ref="G324:G325"/>
+    <mergeCell ref="F326:F329"/>
+    <mergeCell ref="G326:G329"/>
+    <mergeCell ref="G330:G333"/>
+    <mergeCell ref="F330:F333"/>
+    <mergeCell ref="F334:F336"/>
+    <mergeCell ref="F337:F338"/>
+    <mergeCell ref="F339:F340"/>
+    <mergeCell ref="G339:G340"/>
+    <mergeCell ref="F341:F344"/>
+    <mergeCell ref="G341:G344"/>
+    <mergeCell ref="F345:F347"/>
+    <mergeCell ref="G345:G347"/>
+    <mergeCell ref="F348:F349"/>
+    <mergeCell ref="G348:G349"/>
+    <mergeCell ref="F350:F351"/>
+    <mergeCell ref="G350:G351"/>
+    <mergeCell ref="G354:G357"/>
+    <mergeCell ref="F354:F357"/>
+    <mergeCell ref="F358:F359"/>
+    <mergeCell ref="F360:F362"/>
+    <mergeCell ref="F363:F364"/>
+    <mergeCell ref="F365:F368"/>
+    <mergeCell ref="F369:F372"/>
+    <mergeCell ref="F373:F375"/>
+    <mergeCell ref="G358:G359"/>
+    <mergeCell ref="G360:G362"/>
+    <mergeCell ref="G363:G364"/>
+    <mergeCell ref="G365:G368"/>
+    <mergeCell ref="G369:G372"/>
+    <mergeCell ref="G373:G375"/>
+    <mergeCell ref="G376:G377"/>
+    <mergeCell ref="F376:F377"/>
+    <mergeCell ref="F378:F379"/>
+    <mergeCell ref="F380:F383"/>
+    <mergeCell ref="F384:F386"/>
+    <mergeCell ref="F387:F388"/>
+    <mergeCell ref="F389:F390"/>
+    <mergeCell ref="F393:F396"/>
+    <mergeCell ref="F397:F398"/>
+    <mergeCell ref="F399:F401"/>
+    <mergeCell ref="F402:F403"/>
+    <mergeCell ref="F404:F407"/>
+    <mergeCell ref="G404:G407"/>
+    <mergeCell ref="F408:F411"/>
+    <mergeCell ref="G408:G411"/>
     <mergeCell ref="F48:F50"/>
     <mergeCell ref="F85:F86"/>
     <mergeCell ref="G100:G102"/>
@@ -15237,9 +16032,6 @@
     <mergeCell ref="G170:G173"/>
     <mergeCell ref="F207:F208"/>
     <mergeCell ref="G207:G208"/>
-    <mergeCell ref="H241:H242"/>
-    <mergeCell ref="I241:I242"/>
-    <mergeCell ref="J241:J242"/>
     <mergeCell ref="D198:D208"/>
     <mergeCell ref="D209:D219"/>
     <mergeCell ref="D192:D195"/>
@@ -15253,7 +16045,6 @@
     <mergeCell ref="B298:B301"/>
     <mergeCell ref="B302:B308"/>
     <mergeCell ref="B309:B312"/>
-    <mergeCell ref="B326:B336"/>
     <mergeCell ref="E282:E284"/>
     <mergeCell ref="E285:E286"/>
     <mergeCell ref="C287:C297"/>
@@ -15264,15 +16055,9 @@
     <mergeCell ref="C302:C308"/>
     <mergeCell ref="C309:C312"/>
     <mergeCell ref="D309:D312"/>
-    <mergeCell ref="C326:C336"/>
-    <mergeCell ref="D326:D336"/>
     <mergeCell ref="E309:E310"/>
     <mergeCell ref="E311:E312"/>
     <mergeCell ref="E319:E320"/>
-    <mergeCell ref="E321:E323"/>
-    <mergeCell ref="E324:E325"/>
-    <mergeCell ref="E326:E329"/>
-    <mergeCell ref="E330:E333"/>
     <mergeCell ref="C298:C301"/>
     <mergeCell ref="D298:D301"/>
     <mergeCell ref="E298:E299"/>
@@ -15280,21 +16065,8 @@
     <mergeCell ref="D302:D308"/>
     <mergeCell ref="E302:E305"/>
     <mergeCell ref="E306:E308"/>
-    <mergeCell ref="F306:F308"/>
-    <mergeCell ref="F309:F310"/>
-    <mergeCell ref="F311:F312"/>
-    <mergeCell ref="F319:F320"/>
-    <mergeCell ref="F321:F323"/>
-    <mergeCell ref="F324:F325"/>
-    <mergeCell ref="F326:F329"/>
-    <mergeCell ref="F330:F333"/>
-    <mergeCell ref="G309:G310"/>
-    <mergeCell ref="G311:G312"/>
-    <mergeCell ref="G319:G320"/>
-    <mergeCell ref="G321:G323"/>
-    <mergeCell ref="G324:G325"/>
-    <mergeCell ref="G326:G329"/>
-    <mergeCell ref="G330:G333"/>
+    <mergeCell ref="F298:F299"/>
+    <mergeCell ref="G298:G299"/>
     <mergeCell ref="F285:F286"/>
     <mergeCell ref="F287:F290"/>
     <mergeCell ref="G287:G290"/>
@@ -15302,153 +16074,6 @@
     <mergeCell ref="G291:G294"/>
     <mergeCell ref="F295:F297"/>
     <mergeCell ref="G295:G297"/>
-    <mergeCell ref="F315:F318"/>
-    <mergeCell ref="G315:G318"/>
-    <mergeCell ref="F298:F299"/>
-    <mergeCell ref="G298:G299"/>
-    <mergeCell ref="F300:F301"/>
-    <mergeCell ref="G300:G301"/>
-    <mergeCell ref="F302:F305"/>
-    <mergeCell ref="G302:G305"/>
-    <mergeCell ref="G306:G308"/>
-    <mergeCell ref="F454:F455"/>
-    <mergeCell ref="F456:F457"/>
-    <mergeCell ref="G456:G457"/>
-    <mergeCell ref="G447:G450"/>
-    <mergeCell ref="H449:H450"/>
-    <mergeCell ref="I449:I450"/>
-    <mergeCell ref="J449:J450"/>
-    <mergeCell ref="F451:F453"/>
-    <mergeCell ref="G451:G453"/>
-    <mergeCell ref="G454:G455"/>
-    <mergeCell ref="H332:H333"/>
-    <mergeCell ref="I332:I333"/>
-    <mergeCell ref="J332:J333"/>
-    <mergeCell ref="F334:F336"/>
-    <mergeCell ref="G334:G336"/>
-    <mergeCell ref="F337:F338"/>
-    <mergeCell ref="G337:G338"/>
-    <mergeCell ref="H293:H294"/>
-    <mergeCell ref="I293:I294"/>
-    <mergeCell ref="H371:H372"/>
-    <mergeCell ref="I371:I372"/>
-    <mergeCell ref="J371:J372"/>
-    <mergeCell ref="F373:F375"/>
-    <mergeCell ref="G373:G375"/>
-    <mergeCell ref="J358:J359"/>
-    <mergeCell ref="F204:F206"/>
-    <mergeCell ref="G204:G206"/>
-    <mergeCell ref="F174:F177"/>
-    <mergeCell ref="G174:G177"/>
-    <mergeCell ref="F198:F201"/>
-    <mergeCell ref="G198:G201"/>
-    <mergeCell ref="K198:K234"/>
-    <mergeCell ref="F202:F203"/>
-    <mergeCell ref="G202:G203"/>
-    <mergeCell ref="J215:J216"/>
-    <mergeCell ref="K276:K312"/>
-    <mergeCell ref="K315:K351"/>
-    <mergeCell ref="K354:K390"/>
-    <mergeCell ref="K393:K429"/>
-    <mergeCell ref="K432:K468"/>
-    <mergeCell ref="H215:H216"/>
-    <mergeCell ref="I215:I216"/>
-    <mergeCell ref="K237:K273"/>
-    <mergeCell ref="H254:H255"/>
-    <mergeCell ref="I254:I255"/>
-    <mergeCell ref="J254:J255"/>
-    <mergeCell ref="J293:J294"/>
-    <mergeCell ref="F458:F461"/>
-    <mergeCell ref="G458:G461"/>
-    <mergeCell ref="F462:F464"/>
-    <mergeCell ref="G462:G464"/>
-    <mergeCell ref="F465:F466"/>
-    <mergeCell ref="G465:G466"/>
-    <mergeCell ref="F467:F468"/>
-    <mergeCell ref="G467:G468"/>
-    <mergeCell ref="F209:F212"/>
-    <mergeCell ref="G209:G212"/>
-    <mergeCell ref="F280:F281"/>
-    <mergeCell ref="G280:G281"/>
-    <mergeCell ref="F282:F284"/>
-    <mergeCell ref="G282:G284"/>
-    <mergeCell ref="G285:G286"/>
-    <mergeCell ref="H358:H359"/>
-    <mergeCell ref="I358:I359"/>
-    <mergeCell ref="F348:F349"/>
-    <mergeCell ref="F350:F351"/>
-    <mergeCell ref="F354:F357"/>
-    <mergeCell ref="G354:G357"/>
-    <mergeCell ref="F339:F340"/>
-    <mergeCell ref="G339:G340"/>
-    <mergeCell ref="F341:F344"/>
-    <mergeCell ref="G341:G344"/>
-    <mergeCell ref="F345:F347"/>
-    <mergeCell ref="G345:G347"/>
-    <mergeCell ref="G348:G349"/>
-    <mergeCell ref="G350:G351"/>
-    <mergeCell ref="F365:F368"/>
-    <mergeCell ref="F369:F372"/>
-    <mergeCell ref="F358:F359"/>
-    <mergeCell ref="G358:G359"/>
-    <mergeCell ref="F360:F362"/>
-    <mergeCell ref="G360:G362"/>
-    <mergeCell ref="F363:F364"/>
-    <mergeCell ref="G363:G364"/>
-    <mergeCell ref="G365:G368"/>
-    <mergeCell ref="G369:G372"/>
-    <mergeCell ref="F384:F386"/>
-    <mergeCell ref="F387:F388"/>
-    <mergeCell ref="F393:F396"/>
-    <mergeCell ref="G393:G396"/>
-    <mergeCell ref="F376:F377"/>
-    <mergeCell ref="G376:G377"/>
-    <mergeCell ref="F378:F379"/>
-    <mergeCell ref="G378:G379"/>
-    <mergeCell ref="F380:F383"/>
-    <mergeCell ref="G380:G383"/>
-    <mergeCell ref="G384:G386"/>
-    <mergeCell ref="G387:G388"/>
-    <mergeCell ref="F402:F403"/>
-    <mergeCell ref="F404:F407"/>
-    <mergeCell ref="G404:G407"/>
-    <mergeCell ref="F389:F390"/>
-    <mergeCell ref="G389:G390"/>
-    <mergeCell ref="F397:F398"/>
-    <mergeCell ref="G397:G398"/>
-    <mergeCell ref="F399:F401"/>
-    <mergeCell ref="G399:G401"/>
-    <mergeCell ref="G402:G403"/>
-    <mergeCell ref="F415:F416"/>
-    <mergeCell ref="G415:G416"/>
-    <mergeCell ref="F408:F411"/>
-    <mergeCell ref="G408:G411"/>
-    <mergeCell ref="H410:H411"/>
-    <mergeCell ref="I410:I411"/>
-    <mergeCell ref="J410:J411"/>
-    <mergeCell ref="F412:F414"/>
-    <mergeCell ref="G412:G414"/>
-    <mergeCell ref="F426:F427"/>
-    <mergeCell ref="F428:F429"/>
-    <mergeCell ref="F432:F435"/>
-    <mergeCell ref="G432:G435"/>
-    <mergeCell ref="F417:F418"/>
-    <mergeCell ref="G417:G418"/>
-    <mergeCell ref="F419:F422"/>
-    <mergeCell ref="G419:G422"/>
-    <mergeCell ref="F423:F425"/>
-    <mergeCell ref="G423:G425"/>
-    <mergeCell ref="G426:G427"/>
-    <mergeCell ref="G428:G429"/>
-    <mergeCell ref="F443:F446"/>
-    <mergeCell ref="F447:F450"/>
-    <mergeCell ref="F436:F437"/>
-    <mergeCell ref="G436:G437"/>
-    <mergeCell ref="F438:F440"/>
-    <mergeCell ref="G438:G440"/>
-    <mergeCell ref="F441:F442"/>
-    <mergeCell ref="G441:G442"/>
-    <mergeCell ref="G443:G446"/>
   </mergeCells>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -25724,212 +26349,44 @@
     </row>
   </sheetData>
   <mergeCells count="602">
-    <mergeCell ref="F379:F380"/>
-    <mergeCell ref="G379:G380"/>
-    <mergeCell ref="E325:E327"/>
-    <mergeCell ref="F325:F327"/>
-    <mergeCell ref="B377:B380"/>
-    <mergeCell ref="C377:C380"/>
-    <mergeCell ref="D377:D380"/>
-    <mergeCell ref="F377:F378"/>
-    <mergeCell ref="G377:G378"/>
-    <mergeCell ref="E287:E289"/>
-    <mergeCell ref="E290:E291"/>
-    <mergeCell ref="E294:E297"/>
-    <mergeCell ref="F294:F297"/>
-    <mergeCell ref="E298:E300"/>
-    <mergeCell ref="F298:F300"/>
-    <mergeCell ref="F301:F302"/>
-    <mergeCell ref="F303:F304"/>
-    <mergeCell ref="F312:F314"/>
-    <mergeCell ref="G312:G314"/>
-    <mergeCell ref="G315:G316"/>
-    <mergeCell ref="G317:G320"/>
-    <mergeCell ref="G321:G324"/>
-    <mergeCell ref="H323:H324"/>
-    <mergeCell ref="I323:I324"/>
-    <mergeCell ref="J323:J324"/>
-    <mergeCell ref="K344:K380"/>
-    <mergeCell ref="H361:H362"/>
-    <mergeCell ref="I361:I362"/>
-    <mergeCell ref="J361:J362"/>
-    <mergeCell ref="E301:E302"/>
-    <mergeCell ref="E303:E304"/>
-    <mergeCell ref="K306:K342"/>
-    <mergeCell ref="E310:E311"/>
-    <mergeCell ref="F310:F311"/>
-    <mergeCell ref="G310:G311"/>
-    <mergeCell ref="E312:E314"/>
-    <mergeCell ref="E377:E378"/>
-    <mergeCell ref="E379:E380"/>
-    <mergeCell ref="J209:J210"/>
-    <mergeCell ref="H209:H210"/>
-    <mergeCell ref="I209:I210"/>
-    <mergeCell ref="H216:H217"/>
-    <mergeCell ref="I216:I217"/>
-    <mergeCell ref="C180:C186"/>
-    <mergeCell ref="H178:H179"/>
-    <mergeCell ref="I178:I179"/>
-    <mergeCell ref="J178:J179"/>
-    <mergeCell ref="H218:H219"/>
-    <mergeCell ref="I218:I219"/>
-    <mergeCell ref="C154:C164"/>
-    <mergeCell ref="C187:C190"/>
-    <mergeCell ref="C192:C202"/>
-    <mergeCell ref="K192:K228"/>
-    <mergeCell ref="C203:C213"/>
-    <mergeCell ref="G203:G206"/>
-    <mergeCell ref="J216:J217"/>
-    <mergeCell ref="J218:J219"/>
-    <mergeCell ref="D290:D293"/>
-    <mergeCell ref="E292:E293"/>
-    <mergeCell ref="B290:B293"/>
-    <mergeCell ref="B294:B300"/>
-    <mergeCell ref="C294:C300"/>
-    <mergeCell ref="D294:D300"/>
-    <mergeCell ref="B301:B304"/>
-    <mergeCell ref="C301:C304"/>
-    <mergeCell ref="D301:D304"/>
-    <mergeCell ref="D203:D213"/>
-    <mergeCell ref="E207:E210"/>
-    <mergeCell ref="E211:E213"/>
-    <mergeCell ref="F287:F289"/>
-    <mergeCell ref="C290:C293"/>
-    <mergeCell ref="F290:F291"/>
-    <mergeCell ref="F292:F293"/>
-    <mergeCell ref="G292:G293"/>
-    <mergeCell ref="G294:G297"/>
-    <mergeCell ref="G298:G300"/>
-    <mergeCell ref="G301:G302"/>
-    <mergeCell ref="J171:J172"/>
-    <mergeCell ref="H171:H172"/>
-    <mergeCell ref="I171:I172"/>
-    <mergeCell ref="K230:K266"/>
-    <mergeCell ref="J247:J248"/>
-    <mergeCell ref="H247:H248"/>
-    <mergeCell ref="I247:I248"/>
-    <mergeCell ref="K268:K304"/>
-    <mergeCell ref="H285:H286"/>
-    <mergeCell ref="I285:I286"/>
-    <mergeCell ref="J285:J286"/>
-    <mergeCell ref="G287:G289"/>
-    <mergeCell ref="G290:G291"/>
-    <mergeCell ref="G303:G304"/>
-    <mergeCell ref="B241:B251"/>
-    <mergeCell ref="B252:B255"/>
-    <mergeCell ref="C252:C255"/>
-    <mergeCell ref="D252:D255"/>
-    <mergeCell ref="E252:E253"/>
-    <mergeCell ref="F252:F253"/>
-    <mergeCell ref="G252:G253"/>
-    <mergeCell ref="G254:G255"/>
-    <mergeCell ref="F260:F262"/>
-    <mergeCell ref="G260:G262"/>
-    <mergeCell ref="E254:E255"/>
-    <mergeCell ref="F254:F255"/>
-    <mergeCell ref="B256:B262"/>
-    <mergeCell ref="C256:C262"/>
-    <mergeCell ref="D256:D262"/>
-    <mergeCell ref="F256:F259"/>
-    <mergeCell ref="G256:G259"/>
-    <mergeCell ref="D332:D338"/>
-    <mergeCell ref="E336:E338"/>
-    <mergeCell ref="F336:F338"/>
-    <mergeCell ref="G336:G338"/>
-    <mergeCell ref="G306:G309"/>
-    <mergeCell ref="G325:G327"/>
-    <mergeCell ref="G328:G329"/>
-    <mergeCell ref="G330:G331"/>
-    <mergeCell ref="B332:B338"/>
-    <mergeCell ref="C332:C338"/>
-    <mergeCell ref="G332:G335"/>
-    <mergeCell ref="F341:F342"/>
-    <mergeCell ref="G341:G342"/>
-    <mergeCell ref="E332:E335"/>
-    <mergeCell ref="F332:F335"/>
-    <mergeCell ref="B339:B342"/>
-    <mergeCell ref="C339:C342"/>
-    <mergeCell ref="D339:D342"/>
-    <mergeCell ref="F339:F340"/>
-    <mergeCell ref="G339:G340"/>
-    <mergeCell ref="E344:E347"/>
-    <mergeCell ref="E348:E349"/>
-    <mergeCell ref="E350:E352"/>
-    <mergeCell ref="F350:F352"/>
-    <mergeCell ref="D344:D354"/>
-    <mergeCell ref="E353:E354"/>
-    <mergeCell ref="F353:F354"/>
-    <mergeCell ref="G353:G354"/>
-    <mergeCell ref="E339:E340"/>
-    <mergeCell ref="E341:E342"/>
-    <mergeCell ref="B344:B354"/>
-    <mergeCell ref="C344:C354"/>
-    <mergeCell ref="F344:F347"/>
-    <mergeCell ref="G344:G347"/>
-    <mergeCell ref="G350:G352"/>
-    <mergeCell ref="F359:F362"/>
-    <mergeCell ref="G359:G362"/>
-    <mergeCell ref="E363:E365"/>
-    <mergeCell ref="F363:F365"/>
-    <mergeCell ref="F348:F349"/>
-    <mergeCell ref="G348:G349"/>
-    <mergeCell ref="B355:B365"/>
-    <mergeCell ref="C355:C365"/>
-    <mergeCell ref="D355:D365"/>
-    <mergeCell ref="F355:F358"/>
-    <mergeCell ref="G355:G358"/>
-    <mergeCell ref="G363:G365"/>
-    <mergeCell ref="F368:F369"/>
-    <mergeCell ref="G368:G369"/>
-    <mergeCell ref="E355:E358"/>
-    <mergeCell ref="E359:E362"/>
-    <mergeCell ref="B366:B369"/>
-    <mergeCell ref="C366:C369"/>
-    <mergeCell ref="D366:D369"/>
-    <mergeCell ref="F366:F367"/>
-    <mergeCell ref="G366:G367"/>
-    <mergeCell ref="E370:E373"/>
-    <mergeCell ref="E374:E376"/>
-    <mergeCell ref="E366:E367"/>
-    <mergeCell ref="E368:E369"/>
-    <mergeCell ref="B370:B376"/>
-    <mergeCell ref="C370:C376"/>
-    <mergeCell ref="D370:D376"/>
-    <mergeCell ref="F370:F373"/>
-    <mergeCell ref="G370:G373"/>
     <mergeCell ref="F46:F48"/>
     <mergeCell ref="F59:F61"/>
-    <mergeCell ref="H60:H61"/>
-    <mergeCell ref="I60:I61"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="G66:G69"/>
+    <mergeCell ref="F70:F72"/>
+    <mergeCell ref="G70:G72"/>
     <mergeCell ref="F73:F74"/>
     <mergeCell ref="G73:G74"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="G75:G76"/>
+    <mergeCell ref="G82:G83"/>
     <mergeCell ref="F84:F86"/>
     <mergeCell ref="G84:G86"/>
     <mergeCell ref="F87:F88"/>
     <mergeCell ref="G87:G88"/>
+    <mergeCell ref="F44:F45"/>
+    <mergeCell ref="F82:F83"/>
+    <mergeCell ref="F108:F110"/>
+    <mergeCell ref="G108:G110"/>
+    <mergeCell ref="F111:F112"/>
+    <mergeCell ref="G111:G112"/>
+    <mergeCell ref="F113:F114"/>
+    <mergeCell ref="G113:G114"/>
+    <mergeCell ref="F32:F34"/>
+    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="K40:K76"/>
+    <mergeCell ref="G44:G45"/>
+    <mergeCell ref="G46:G48"/>
+    <mergeCell ref="J57:J58"/>
+    <mergeCell ref="K78:K114"/>
     <mergeCell ref="F89:F92"/>
     <mergeCell ref="G89:G92"/>
     <mergeCell ref="F93:F96"/>
     <mergeCell ref="G93:G96"/>
     <mergeCell ref="H95:H96"/>
     <mergeCell ref="I95:I96"/>
-    <mergeCell ref="F82:F83"/>
+    <mergeCell ref="J95:J96"/>
     <mergeCell ref="F97:F99"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="G75:G76"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="G78:G81"/>
-    <mergeCell ref="K78:K114"/>
-    <mergeCell ref="G82:G83"/>
-    <mergeCell ref="J95:J96"/>
-    <mergeCell ref="F32:F34"/>
-    <mergeCell ref="G32:G34"/>
-    <mergeCell ref="K40:K76"/>
-    <mergeCell ref="F44:F45"/>
-    <mergeCell ref="G44:G45"/>
-    <mergeCell ref="G46:G48"/>
-    <mergeCell ref="J57:J58"/>
-    <mergeCell ref="J60:J61"/>
     <mergeCell ref="G97:G99"/>
     <mergeCell ref="F100:F101"/>
     <mergeCell ref="G100:G101"/>
@@ -25937,37 +26394,127 @@
     <mergeCell ref="G102:G103"/>
     <mergeCell ref="F104:F107"/>
     <mergeCell ref="G104:G107"/>
-    <mergeCell ref="F108:F110"/>
-    <mergeCell ref="G108:G110"/>
-    <mergeCell ref="F111:F112"/>
-    <mergeCell ref="G111:G112"/>
-    <mergeCell ref="F113:F114"/>
-    <mergeCell ref="G113:G114"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="B28:B34"/>
-    <mergeCell ref="C28:C34"/>
-    <mergeCell ref="D28:D34"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="E32:E34"/>
-    <mergeCell ref="F28:F31"/>
-    <mergeCell ref="G28:G31"/>
-    <mergeCell ref="D35:D38"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="D40:D50"/>
-    <mergeCell ref="E40:E43"/>
-    <mergeCell ref="F40:F43"/>
-    <mergeCell ref="G40:G43"/>
-    <mergeCell ref="E44:E45"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="E62:E63"/>
-    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="E169:E172"/>
+    <mergeCell ref="E173:E175"/>
+    <mergeCell ref="E120:E121"/>
+    <mergeCell ref="E122:E124"/>
+    <mergeCell ref="E154:E157"/>
+    <mergeCell ref="E158:E159"/>
+    <mergeCell ref="E160:E162"/>
+    <mergeCell ref="E163:E164"/>
+    <mergeCell ref="E165:E168"/>
+    <mergeCell ref="D116:D126"/>
+    <mergeCell ref="D154:D164"/>
+    <mergeCell ref="D165:D175"/>
+    <mergeCell ref="D176:D179"/>
+    <mergeCell ref="D180:D186"/>
+    <mergeCell ref="D187:D190"/>
+    <mergeCell ref="D192:D202"/>
+    <mergeCell ref="D203:D213"/>
+    <mergeCell ref="D214:D217"/>
+    <mergeCell ref="D218:D224"/>
+    <mergeCell ref="D225:D228"/>
+    <mergeCell ref="D230:D240"/>
+    <mergeCell ref="D241:D251"/>
+    <mergeCell ref="D252:D255"/>
+    <mergeCell ref="D256:D262"/>
+    <mergeCell ref="D263:D266"/>
+    <mergeCell ref="D268:D278"/>
+    <mergeCell ref="D279:D289"/>
+    <mergeCell ref="D290:D293"/>
+    <mergeCell ref="D294:D300"/>
+    <mergeCell ref="D301:D304"/>
+    <mergeCell ref="D366:D369"/>
+    <mergeCell ref="D370:D376"/>
+    <mergeCell ref="D377:D380"/>
+    <mergeCell ref="D306:D316"/>
+    <mergeCell ref="D317:D327"/>
+    <mergeCell ref="D328:D331"/>
+    <mergeCell ref="D332:D338"/>
+    <mergeCell ref="D339:D342"/>
+    <mergeCell ref="D344:D354"/>
+    <mergeCell ref="D355:D365"/>
+    <mergeCell ref="C78:C88"/>
+    <mergeCell ref="B89:B99"/>
+    <mergeCell ref="C89:C99"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="C35:C38"/>
+    <mergeCell ref="A40:A76"/>
+    <mergeCell ref="B40:B50"/>
+    <mergeCell ref="C40:C50"/>
+    <mergeCell ref="C51:C61"/>
+    <mergeCell ref="A78:A114"/>
+    <mergeCell ref="B180:B186"/>
+    <mergeCell ref="C180:C186"/>
+    <mergeCell ref="B187:B190"/>
+    <mergeCell ref="C187:C190"/>
+    <mergeCell ref="B176:B179"/>
+    <mergeCell ref="B192:B202"/>
+    <mergeCell ref="B214:B217"/>
+    <mergeCell ref="C214:C217"/>
+    <mergeCell ref="B218:B224"/>
+    <mergeCell ref="C218:C224"/>
+    <mergeCell ref="E189:E190"/>
+    <mergeCell ref="E192:E195"/>
+    <mergeCell ref="E196:E197"/>
+    <mergeCell ref="E198:E200"/>
+    <mergeCell ref="E201:E202"/>
+    <mergeCell ref="E203:E206"/>
+    <mergeCell ref="E207:E210"/>
+    <mergeCell ref="E211:E213"/>
+    <mergeCell ref="E214:E215"/>
+    <mergeCell ref="E216:E217"/>
+    <mergeCell ref="E218:E221"/>
+    <mergeCell ref="E222:E224"/>
+    <mergeCell ref="E225:E226"/>
+    <mergeCell ref="E227:E228"/>
+    <mergeCell ref="E252:E253"/>
+    <mergeCell ref="E254:E255"/>
+    <mergeCell ref="E256:E259"/>
+    <mergeCell ref="E260:E262"/>
+    <mergeCell ref="E263:E264"/>
+    <mergeCell ref="E265:E266"/>
+    <mergeCell ref="E268:E271"/>
+    <mergeCell ref="E272:E273"/>
+    <mergeCell ref="E274:E276"/>
+    <mergeCell ref="E277:E278"/>
+    <mergeCell ref="E279:E282"/>
+    <mergeCell ref="E283:E286"/>
+    <mergeCell ref="E287:E289"/>
+    <mergeCell ref="E290:E291"/>
+    <mergeCell ref="E292:E293"/>
+    <mergeCell ref="E294:E297"/>
+    <mergeCell ref="E298:E300"/>
+    <mergeCell ref="E301:E302"/>
+    <mergeCell ref="E303:E304"/>
+    <mergeCell ref="E306:E309"/>
+    <mergeCell ref="E310:E311"/>
+    <mergeCell ref="E312:E314"/>
+    <mergeCell ref="E315:E316"/>
+    <mergeCell ref="E317:E320"/>
+    <mergeCell ref="E321:E324"/>
+    <mergeCell ref="E325:E327"/>
+    <mergeCell ref="E328:E329"/>
+    <mergeCell ref="E330:E331"/>
+    <mergeCell ref="E332:E335"/>
+    <mergeCell ref="E336:E338"/>
+    <mergeCell ref="E339:E340"/>
+    <mergeCell ref="E341:E342"/>
+    <mergeCell ref="E344:E347"/>
+    <mergeCell ref="E348:E349"/>
+    <mergeCell ref="E350:E352"/>
+    <mergeCell ref="E374:E376"/>
+    <mergeCell ref="E377:E378"/>
+    <mergeCell ref="E379:E380"/>
+    <mergeCell ref="E353:E354"/>
+    <mergeCell ref="E355:E358"/>
+    <mergeCell ref="E359:E362"/>
+    <mergeCell ref="E363:E365"/>
+    <mergeCell ref="E366:E367"/>
+    <mergeCell ref="E368:E369"/>
+    <mergeCell ref="E370:E373"/>
     <mergeCell ref="E66:E69"/>
     <mergeCell ref="E70:E72"/>
-    <mergeCell ref="F70:F72"/>
-    <mergeCell ref="G70:G72"/>
     <mergeCell ref="E46:E48"/>
     <mergeCell ref="E49:E50"/>
     <mergeCell ref="D51:D61"/>
@@ -25975,216 +26522,92 @@
     <mergeCell ref="E55:E58"/>
     <mergeCell ref="E59:E61"/>
     <mergeCell ref="D66:D72"/>
+    <mergeCell ref="E93:E96"/>
+    <mergeCell ref="E97:E99"/>
     <mergeCell ref="D78:D88"/>
-    <mergeCell ref="D89:D99"/>
-    <mergeCell ref="D100:D103"/>
-    <mergeCell ref="D104:D110"/>
-    <mergeCell ref="D111:D114"/>
-    <mergeCell ref="D116:D126"/>
-    <mergeCell ref="D73:D76"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="E75:E76"/>
     <mergeCell ref="E78:E81"/>
     <mergeCell ref="E82:E83"/>
     <mergeCell ref="E84:E86"/>
     <mergeCell ref="E87:E88"/>
+    <mergeCell ref="D89:D99"/>
     <mergeCell ref="E89:E92"/>
-    <mergeCell ref="E93:E96"/>
-    <mergeCell ref="E97:E99"/>
+    <mergeCell ref="D100:D103"/>
     <mergeCell ref="E100:E101"/>
     <mergeCell ref="E102:E103"/>
+    <mergeCell ref="D104:D110"/>
     <mergeCell ref="E104:E107"/>
-    <mergeCell ref="E108:E110"/>
-    <mergeCell ref="F120:F121"/>
-    <mergeCell ref="G120:G121"/>
-    <mergeCell ref="E122:E124"/>
-    <mergeCell ref="F122:F124"/>
-    <mergeCell ref="F125:F126"/>
-    <mergeCell ref="G125:G126"/>
-    <mergeCell ref="F116:F119"/>
-    <mergeCell ref="F135:F137"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="G142:G145"/>
-    <mergeCell ref="E146:E148"/>
-    <mergeCell ref="F146:F148"/>
-    <mergeCell ref="G146:G148"/>
-    <mergeCell ref="E149:E150"/>
-    <mergeCell ref="F149:F150"/>
-    <mergeCell ref="G149:G150"/>
-    <mergeCell ref="E151:E152"/>
-    <mergeCell ref="F151:F152"/>
-    <mergeCell ref="G151:G152"/>
-    <mergeCell ref="F158:F159"/>
-    <mergeCell ref="G158:G159"/>
-    <mergeCell ref="E160:E162"/>
-    <mergeCell ref="F160:F162"/>
-    <mergeCell ref="E116:E119"/>
-    <mergeCell ref="E158:E159"/>
-    <mergeCell ref="F180:F183"/>
-    <mergeCell ref="G180:G183"/>
-    <mergeCell ref="E184:E186"/>
-    <mergeCell ref="F184:F186"/>
-    <mergeCell ref="G184:G186"/>
-    <mergeCell ref="E187:E188"/>
-    <mergeCell ref="F187:F188"/>
-    <mergeCell ref="G187:G188"/>
-    <mergeCell ref="E189:E190"/>
-    <mergeCell ref="F189:F190"/>
+    <mergeCell ref="D111:D114"/>
+    <mergeCell ref="E125:E126"/>
     <mergeCell ref="E111:E112"/>
     <mergeCell ref="E113:E114"/>
-    <mergeCell ref="G116:G119"/>
-    <mergeCell ref="K116:K152"/>
-    <mergeCell ref="G122:G124"/>
-    <mergeCell ref="J133:J134"/>
-    <mergeCell ref="K154:K190"/>
-    <mergeCell ref="G189:G190"/>
-    <mergeCell ref="G160:G162"/>
-    <mergeCell ref="E163:E164"/>
-    <mergeCell ref="F163:F164"/>
-    <mergeCell ref="G163:G164"/>
-    <mergeCell ref="E165:E168"/>
-    <mergeCell ref="F165:F168"/>
-    <mergeCell ref="G165:G168"/>
-    <mergeCell ref="E169:E172"/>
-    <mergeCell ref="F169:F172"/>
-    <mergeCell ref="G169:G172"/>
-    <mergeCell ref="E173:E175"/>
-    <mergeCell ref="F173:F175"/>
-    <mergeCell ref="G173:G175"/>
     <mergeCell ref="E176:E177"/>
-    <mergeCell ref="F176:F177"/>
-    <mergeCell ref="G176:G177"/>
     <mergeCell ref="E178:E179"/>
-    <mergeCell ref="F178:F179"/>
-    <mergeCell ref="G178:G179"/>
     <mergeCell ref="E180:E183"/>
-    <mergeCell ref="E120:E121"/>
-    <mergeCell ref="E125:E126"/>
-    <mergeCell ref="D127:D137"/>
-    <mergeCell ref="E127:E130"/>
-    <mergeCell ref="E131:E134"/>
-    <mergeCell ref="E135:E137"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="D142:D148"/>
-    <mergeCell ref="D149:D152"/>
-    <mergeCell ref="D154:D164"/>
-    <mergeCell ref="D165:D175"/>
-    <mergeCell ref="D176:D179"/>
-    <mergeCell ref="D180:D186"/>
-    <mergeCell ref="D187:D190"/>
-    <mergeCell ref="E196:E197"/>
-    <mergeCell ref="E201:E202"/>
-    <mergeCell ref="F201:F202"/>
-    <mergeCell ref="G201:G202"/>
-    <mergeCell ref="D192:D202"/>
-    <mergeCell ref="E192:E195"/>
-    <mergeCell ref="F192:F195"/>
-    <mergeCell ref="G192:G195"/>
-    <mergeCell ref="F196:F197"/>
-    <mergeCell ref="G196:G197"/>
-    <mergeCell ref="G198:G200"/>
-    <mergeCell ref="F127:F130"/>
-    <mergeCell ref="G127:G130"/>
-    <mergeCell ref="F131:F134"/>
-    <mergeCell ref="G131:G134"/>
-    <mergeCell ref="H133:H134"/>
-    <mergeCell ref="I133:I134"/>
-    <mergeCell ref="G135:G137"/>
-    <mergeCell ref="F138:F139"/>
-    <mergeCell ref="G138:G139"/>
-    <mergeCell ref="E138:E139"/>
-    <mergeCell ref="E140:E141"/>
-    <mergeCell ref="E154:E157"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="G154:G157"/>
-    <mergeCell ref="F140:F141"/>
-    <mergeCell ref="G140:G141"/>
-    <mergeCell ref="E198:E200"/>
-    <mergeCell ref="F198:F200"/>
-    <mergeCell ref="C214:C217"/>
-    <mergeCell ref="D214:D217"/>
-    <mergeCell ref="E214:E215"/>
-    <mergeCell ref="F214:F215"/>
-    <mergeCell ref="G214:G215"/>
-    <mergeCell ref="E216:E217"/>
-    <mergeCell ref="F216:F217"/>
-    <mergeCell ref="G216:G217"/>
-    <mergeCell ref="C218:C224"/>
-    <mergeCell ref="D218:D224"/>
-    <mergeCell ref="E218:E221"/>
-    <mergeCell ref="F218:F221"/>
-    <mergeCell ref="G218:G221"/>
-    <mergeCell ref="E222:E224"/>
-    <mergeCell ref="F222:F224"/>
-    <mergeCell ref="G222:G224"/>
+    <mergeCell ref="E184:E186"/>
+    <mergeCell ref="E187:E188"/>
+    <mergeCell ref="E230:E233"/>
+    <mergeCell ref="E234:E235"/>
+    <mergeCell ref="E236:E238"/>
+    <mergeCell ref="E239:E240"/>
+    <mergeCell ref="E241:E244"/>
+    <mergeCell ref="E245:E248"/>
+    <mergeCell ref="E249:E251"/>
+    <mergeCell ref="B290:B293"/>
+    <mergeCell ref="B294:B300"/>
+    <mergeCell ref="C294:C300"/>
+    <mergeCell ref="C301:C304"/>
+    <mergeCell ref="C306:C316"/>
+    <mergeCell ref="B306:B316"/>
+    <mergeCell ref="B317:B327"/>
+    <mergeCell ref="C317:C327"/>
+    <mergeCell ref="B328:B331"/>
+    <mergeCell ref="C328:C331"/>
+    <mergeCell ref="B332:B338"/>
+    <mergeCell ref="C332:C338"/>
+    <mergeCell ref="C192:C202"/>
+    <mergeCell ref="B203:B213"/>
+    <mergeCell ref="C203:C213"/>
+    <mergeCell ref="B225:B228"/>
     <mergeCell ref="C225:C228"/>
-    <mergeCell ref="D225:D228"/>
-    <mergeCell ref="E203:E206"/>
-    <mergeCell ref="F203:F206"/>
-    <mergeCell ref="E225:E226"/>
-    <mergeCell ref="F225:F226"/>
-    <mergeCell ref="G225:G226"/>
-    <mergeCell ref="F227:F228"/>
-    <mergeCell ref="G227:G228"/>
-    <mergeCell ref="E227:E228"/>
-    <mergeCell ref="E230:E233"/>
-    <mergeCell ref="F230:F233"/>
-    <mergeCell ref="G230:G233"/>
-    <mergeCell ref="E234:E235"/>
-    <mergeCell ref="F234:F235"/>
-    <mergeCell ref="G234:G235"/>
-    <mergeCell ref="F241:F244"/>
-    <mergeCell ref="G241:G244"/>
-    <mergeCell ref="E236:E238"/>
-    <mergeCell ref="F236:F238"/>
-    <mergeCell ref="G236:G238"/>
-    <mergeCell ref="E239:E240"/>
-    <mergeCell ref="F239:F240"/>
-    <mergeCell ref="G239:G240"/>
-    <mergeCell ref="E241:E244"/>
-    <mergeCell ref="E249:E251"/>
-    <mergeCell ref="F249:F251"/>
-    <mergeCell ref="B230:B240"/>
+    <mergeCell ref="C230:C240"/>
     <mergeCell ref="C241:C251"/>
-    <mergeCell ref="D241:D251"/>
-    <mergeCell ref="E245:E248"/>
-    <mergeCell ref="F245:F248"/>
-    <mergeCell ref="G245:G248"/>
-    <mergeCell ref="G249:G251"/>
-    <mergeCell ref="F265:F266"/>
-    <mergeCell ref="G265:G266"/>
-    <mergeCell ref="E256:E259"/>
-    <mergeCell ref="E260:E262"/>
-    <mergeCell ref="B263:B266"/>
+    <mergeCell ref="C252:C255"/>
+    <mergeCell ref="C256:C262"/>
     <mergeCell ref="C263:C266"/>
-    <mergeCell ref="D263:D266"/>
-    <mergeCell ref="F263:F264"/>
-    <mergeCell ref="G263:G264"/>
-    <mergeCell ref="E268:E271"/>
-    <mergeCell ref="E272:E273"/>
-    <mergeCell ref="E274:E276"/>
-    <mergeCell ref="F274:F276"/>
-    <mergeCell ref="D268:D278"/>
-    <mergeCell ref="E277:E278"/>
-    <mergeCell ref="F277:F278"/>
-    <mergeCell ref="G277:G278"/>
-    <mergeCell ref="E263:E264"/>
-    <mergeCell ref="E265:E266"/>
+    <mergeCell ref="C268:C278"/>
+    <mergeCell ref="A154:A190"/>
+    <mergeCell ref="B154:B164"/>
+    <mergeCell ref="C154:C164"/>
+    <mergeCell ref="B165:B175"/>
+    <mergeCell ref="C165:C175"/>
+    <mergeCell ref="C176:C179"/>
+    <mergeCell ref="A192:A228"/>
     <mergeCell ref="B268:B278"/>
-    <mergeCell ref="C268:C278"/>
-    <mergeCell ref="F268:F271"/>
-    <mergeCell ref="G268:G271"/>
-    <mergeCell ref="G274:G276"/>
-    <mergeCell ref="F283:F286"/>
-    <mergeCell ref="G283:G286"/>
-    <mergeCell ref="F272:F273"/>
-    <mergeCell ref="G272:G273"/>
     <mergeCell ref="B279:B289"/>
     <mergeCell ref="C279:C289"/>
-    <mergeCell ref="D279:D289"/>
-    <mergeCell ref="F279:F282"/>
-    <mergeCell ref="G279:G282"/>
+    <mergeCell ref="C290:C293"/>
+    <mergeCell ref="A268:A304"/>
+    <mergeCell ref="A306:A342"/>
+    <mergeCell ref="A344:A380"/>
+    <mergeCell ref="A230:A266"/>
+    <mergeCell ref="B230:B240"/>
+    <mergeCell ref="B241:B251"/>
+    <mergeCell ref="B252:B255"/>
+    <mergeCell ref="B256:B262"/>
+    <mergeCell ref="B263:B266"/>
+    <mergeCell ref="B301:B304"/>
+    <mergeCell ref="B366:B369"/>
+    <mergeCell ref="B370:B376"/>
+    <mergeCell ref="C370:C376"/>
+    <mergeCell ref="B377:B380"/>
+    <mergeCell ref="C377:C380"/>
+    <mergeCell ref="B339:B342"/>
+    <mergeCell ref="C339:C342"/>
+    <mergeCell ref="B344:B354"/>
+    <mergeCell ref="C344:C354"/>
+    <mergeCell ref="B355:B365"/>
+    <mergeCell ref="C355:C365"/>
+    <mergeCell ref="C366:C369"/>
     <mergeCell ref="E2:E5"/>
     <mergeCell ref="E6:E7"/>
     <mergeCell ref="F6:F7"/>
@@ -26238,22 +26661,39 @@
     <mergeCell ref="H57:H58"/>
     <mergeCell ref="I57:I58"/>
     <mergeCell ref="G59:G61"/>
+    <mergeCell ref="H60:H61"/>
+    <mergeCell ref="I60:I61"/>
+    <mergeCell ref="J60:J61"/>
     <mergeCell ref="F62:F63"/>
     <mergeCell ref="G62:G63"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="B28:B34"/>
+    <mergeCell ref="C28:C34"/>
+    <mergeCell ref="D28:D34"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="F28:F31"/>
+    <mergeCell ref="G28:G31"/>
+    <mergeCell ref="D35:D38"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="D40:D50"/>
+    <mergeCell ref="E40:E43"/>
+    <mergeCell ref="F40:F43"/>
+    <mergeCell ref="G40:G43"/>
+    <mergeCell ref="E44:E45"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="E62:E63"/>
+    <mergeCell ref="E64:E65"/>
     <mergeCell ref="F64:F65"/>
     <mergeCell ref="G64:G65"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="G66:G69"/>
-    <mergeCell ref="C78:C88"/>
-    <mergeCell ref="B89:B99"/>
-    <mergeCell ref="C89:C99"/>
-    <mergeCell ref="B35:B38"/>
-    <mergeCell ref="C35:C38"/>
-    <mergeCell ref="A40:A76"/>
-    <mergeCell ref="B40:B50"/>
-    <mergeCell ref="C40:C50"/>
-    <mergeCell ref="C51:C61"/>
-    <mergeCell ref="A78:A114"/>
+    <mergeCell ref="D73:D76"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="G78:G81"/>
     <mergeCell ref="B66:B72"/>
     <mergeCell ref="C66:C72"/>
     <mergeCell ref="B73:B76"/>
@@ -26264,35 +26704,6 @@
     <mergeCell ref="C100:C103"/>
     <mergeCell ref="B104:B110"/>
     <mergeCell ref="C104:C110"/>
-    <mergeCell ref="B154:B164"/>
-    <mergeCell ref="B165:B175"/>
-    <mergeCell ref="C165:C175"/>
-    <mergeCell ref="C176:C179"/>
-    <mergeCell ref="B176:B179"/>
-    <mergeCell ref="B180:B186"/>
-    <mergeCell ref="E321:E324"/>
-    <mergeCell ref="F321:F324"/>
-    <mergeCell ref="E315:E316"/>
-    <mergeCell ref="F315:F316"/>
-    <mergeCell ref="B317:B327"/>
-    <mergeCell ref="C317:C327"/>
-    <mergeCell ref="D317:D327"/>
-    <mergeCell ref="E317:E320"/>
-    <mergeCell ref="F317:F320"/>
-    <mergeCell ref="B328:B331"/>
-    <mergeCell ref="C328:C331"/>
-    <mergeCell ref="D328:D331"/>
-    <mergeCell ref="E328:E329"/>
-    <mergeCell ref="F328:F329"/>
-    <mergeCell ref="E330:E331"/>
-    <mergeCell ref="F330:F331"/>
-    <mergeCell ref="E279:E282"/>
-    <mergeCell ref="E283:E286"/>
-    <mergeCell ref="B306:B316"/>
-    <mergeCell ref="C306:C316"/>
-    <mergeCell ref="D306:D316"/>
-    <mergeCell ref="E306:E309"/>
-    <mergeCell ref="F306:F309"/>
     <mergeCell ref="B111:B114"/>
     <mergeCell ref="C111:C114"/>
     <mergeCell ref="C116:C126"/>
@@ -26300,31 +26711,245 @@
     <mergeCell ref="C138:C141"/>
     <mergeCell ref="C142:C148"/>
     <mergeCell ref="C149:C152"/>
-    <mergeCell ref="A154:A190"/>
-    <mergeCell ref="A192:A228"/>
-    <mergeCell ref="A230:A266"/>
-    <mergeCell ref="A268:A304"/>
-    <mergeCell ref="A306:A342"/>
-    <mergeCell ref="A344:A380"/>
     <mergeCell ref="A116:A152"/>
     <mergeCell ref="B116:B126"/>
     <mergeCell ref="B127:B137"/>
     <mergeCell ref="B138:B141"/>
     <mergeCell ref="B142:B148"/>
     <mergeCell ref="B149:B152"/>
-    <mergeCell ref="B187:B190"/>
+    <mergeCell ref="F122:F124"/>
+    <mergeCell ref="G122:G124"/>
+    <mergeCell ref="F125:F126"/>
+    <mergeCell ref="G125:G126"/>
+    <mergeCell ref="D127:D137"/>
+    <mergeCell ref="E127:E130"/>
+    <mergeCell ref="E131:E134"/>
+    <mergeCell ref="E135:E137"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="E138:E139"/>
+    <mergeCell ref="D142:D148"/>
+    <mergeCell ref="D149:D152"/>
+    <mergeCell ref="F127:F130"/>
+    <mergeCell ref="G127:G130"/>
+    <mergeCell ref="F131:F134"/>
+    <mergeCell ref="G131:G134"/>
+    <mergeCell ref="H133:H134"/>
+    <mergeCell ref="I133:I134"/>
+    <mergeCell ref="G135:G137"/>
+    <mergeCell ref="F138:F139"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="G154:G157"/>
+    <mergeCell ref="G265:G266"/>
+    <mergeCell ref="G268:G271"/>
+    <mergeCell ref="G272:G273"/>
+    <mergeCell ref="G274:G276"/>
+    <mergeCell ref="G277:G278"/>
+    <mergeCell ref="G279:G282"/>
+    <mergeCell ref="G283:G286"/>
+    <mergeCell ref="G287:G289"/>
+    <mergeCell ref="G290:G291"/>
+    <mergeCell ref="G292:G293"/>
+    <mergeCell ref="G294:G297"/>
+    <mergeCell ref="G298:G300"/>
+    <mergeCell ref="G301:G302"/>
+    <mergeCell ref="G303:G304"/>
+    <mergeCell ref="F234:F235"/>
+    <mergeCell ref="G234:G235"/>
+    <mergeCell ref="F236:F238"/>
+    <mergeCell ref="G236:G238"/>
+    <mergeCell ref="F239:F240"/>
+    <mergeCell ref="G239:G240"/>
+    <mergeCell ref="G241:G244"/>
+    <mergeCell ref="F241:F244"/>
+    <mergeCell ref="F245:F248"/>
+    <mergeCell ref="F249:F251"/>
+    <mergeCell ref="F252:F253"/>
+    <mergeCell ref="F254:F255"/>
+    <mergeCell ref="F256:F259"/>
+    <mergeCell ref="F260:F262"/>
+    <mergeCell ref="G245:G248"/>
+    <mergeCell ref="G249:G251"/>
+    <mergeCell ref="G252:G253"/>
+    <mergeCell ref="G254:G255"/>
+    <mergeCell ref="G256:G259"/>
+    <mergeCell ref="G260:G262"/>
+    <mergeCell ref="G263:G264"/>
+    <mergeCell ref="F263:F264"/>
+    <mergeCell ref="F265:F266"/>
+    <mergeCell ref="F268:F271"/>
+    <mergeCell ref="F272:F273"/>
+    <mergeCell ref="F274:F276"/>
+    <mergeCell ref="F277:F278"/>
+    <mergeCell ref="F279:F282"/>
+    <mergeCell ref="F283:F286"/>
+    <mergeCell ref="F287:F289"/>
+    <mergeCell ref="F290:F291"/>
+    <mergeCell ref="F292:F293"/>
+    <mergeCell ref="F294:F297"/>
+    <mergeCell ref="F298:F300"/>
+    <mergeCell ref="F301:F302"/>
+    <mergeCell ref="F325:F327"/>
+    <mergeCell ref="F328:F329"/>
+    <mergeCell ref="F330:F331"/>
+    <mergeCell ref="F344:F347"/>
+    <mergeCell ref="G344:G347"/>
+    <mergeCell ref="F303:F304"/>
+    <mergeCell ref="F306:F309"/>
+    <mergeCell ref="F310:F311"/>
+    <mergeCell ref="F312:F314"/>
+    <mergeCell ref="F315:F316"/>
+    <mergeCell ref="F317:F320"/>
+    <mergeCell ref="F321:F324"/>
+    <mergeCell ref="F120:F121"/>
+    <mergeCell ref="F135:F137"/>
+    <mergeCell ref="G138:G139"/>
+    <mergeCell ref="E140:E141"/>
+    <mergeCell ref="F140:F141"/>
+    <mergeCell ref="G140:G141"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="G142:G145"/>
+    <mergeCell ref="E146:E148"/>
+    <mergeCell ref="F146:F148"/>
+    <mergeCell ref="G146:G148"/>
+    <mergeCell ref="E149:E150"/>
+    <mergeCell ref="F149:F150"/>
+    <mergeCell ref="G149:G150"/>
+    <mergeCell ref="E151:E152"/>
+    <mergeCell ref="F151:F152"/>
+    <mergeCell ref="G151:G152"/>
+    <mergeCell ref="G158:G159"/>
+    <mergeCell ref="F160:F162"/>
+    <mergeCell ref="G160:G162"/>
+    <mergeCell ref="F163:F164"/>
+    <mergeCell ref="G163:G164"/>
+    <mergeCell ref="F165:F168"/>
+    <mergeCell ref="G165:G168"/>
+    <mergeCell ref="F169:F172"/>
+    <mergeCell ref="G169:G172"/>
+    <mergeCell ref="H171:H172"/>
+    <mergeCell ref="I171:I172"/>
+    <mergeCell ref="J171:J172"/>
+    <mergeCell ref="F173:F175"/>
+    <mergeCell ref="G173:G175"/>
+    <mergeCell ref="F176:F177"/>
+    <mergeCell ref="G176:G177"/>
+    <mergeCell ref="F178:F179"/>
+    <mergeCell ref="G178:G179"/>
+    <mergeCell ref="F187:F188"/>
+    <mergeCell ref="G187:G188"/>
+    <mergeCell ref="F189:F190"/>
+    <mergeCell ref="G189:G190"/>
+    <mergeCell ref="F192:F195"/>
+    <mergeCell ref="G192:G195"/>
+    <mergeCell ref="F196:F197"/>
+    <mergeCell ref="G196:G197"/>
+    <mergeCell ref="G198:G200"/>
+    <mergeCell ref="K192:K228"/>
+    <mergeCell ref="K230:K266"/>
+    <mergeCell ref="K268:K304"/>
+    <mergeCell ref="K306:K342"/>
+    <mergeCell ref="K344:K380"/>
+    <mergeCell ref="H178:H179"/>
+    <mergeCell ref="I178:I179"/>
+    <mergeCell ref="H209:H210"/>
+    <mergeCell ref="I209:I210"/>
+    <mergeCell ref="J209:J210"/>
+    <mergeCell ref="H216:H217"/>
+    <mergeCell ref="J218:J219"/>
+    <mergeCell ref="H285:H286"/>
+    <mergeCell ref="H323:H324"/>
+    <mergeCell ref="I323:I324"/>
+    <mergeCell ref="J323:J324"/>
+    <mergeCell ref="H361:H362"/>
+    <mergeCell ref="I361:I362"/>
+    <mergeCell ref="J361:J362"/>
+    <mergeCell ref="H218:H219"/>
+    <mergeCell ref="I218:I219"/>
+    <mergeCell ref="H247:H248"/>
+    <mergeCell ref="I247:I248"/>
+    <mergeCell ref="J247:J248"/>
+    <mergeCell ref="I285:I286"/>
+    <mergeCell ref="J285:J286"/>
+    <mergeCell ref="G222:G224"/>
+    <mergeCell ref="G225:G226"/>
+    <mergeCell ref="G201:G202"/>
+    <mergeCell ref="G203:G206"/>
+    <mergeCell ref="G207:G210"/>
+    <mergeCell ref="G211:G213"/>
+    <mergeCell ref="G214:G215"/>
+    <mergeCell ref="G216:G217"/>
+    <mergeCell ref="G218:G221"/>
+    <mergeCell ref="F116:F119"/>
+    <mergeCell ref="F158:F159"/>
+    <mergeCell ref="J178:J179"/>
+    <mergeCell ref="F180:F183"/>
+    <mergeCell ref="G180:G183"/>
+    <mergeCell ref="F184:F186"/>
+    <mergeCell ref="G184:G186"/>
+    <mergeCell ref="E108:E110"/>
+    <mergeCell ref="E116:E119"/>
+    <mergeCell ref="G116:G119"/>
+    <mergeCell ref="K116:K152"/>
+    <mergeCell ref="G120:G121"/>
+    <mergeCell ref="J133:J134"/>
+    <mergeCell ref="K154:K190"/>
+    <mergeCell ref="I216:I217"/>
+    <mergeCell ref="J216:J217"/>
+    <mergeCell ref="F198:F200"/>
+    <mergeCell ref="F201:F202"/>
+    <mergeCell ref="F203:F206"/>
     <mergeCell ref="F207:F210"/>
-    <mergeCell ref="G207:G210"/>
     <mergeCell ref="F211:F213"/>
-    <mergeCell ref="G211:G213"/>
-    <mergeCell ref="B192:B202"/>
-    <mergeCell ref="B203:B213"/>
-    <mergeCell ref="B214:B217"/>
-    <mergeCell ref="B218:B224"/>
-    <mergeCell ref="B225:B228"/>
-    <mergeCell ref="C230:C240"/>
-    <mergeCell ref="D230:D240"/>
+    <mergeCell ref="F214:F215"/>
+    <mergeCell ref="F216:F217"/>
+    <mergeCell ref="F218:F221"/>
+    <mergeCell ref="F222:F224"/>
+    <mergeCell ref="F225:F226"/>
+    <mergeCell ref="F227:F228"/>
+    <mergeCell ref="G227:G228"/>
+    <mergeCell ref="F230:F233"/>
+    <mergeCell ref="G230:G233"/>
+    <mergeCell ref="G306:G309"/>
+    <mergeCell ref="G310:G311"/>
+    <mergeCell ref="G312:G314"/>
+    <mergeCell ref="G315:G316"/>
+    <mergeCell ref="G317:G320"/>
+    <mergeCell ref="G321:G324"/>
+    <mergeCell ref="G325:G327"/>
+    <mergeCell ref="G328:G329"/>
+    <mergeCell ref="G330:G331"/>
+    <mergeCell ref="F332:F335"/>
+    <mergeCell ref="G332:G335"/>
+    <mergeCell ref="F336:F338"/>
+    <mergeCell ref="G336:G338"/>
+    <mergeCell ref="G339:G340"/>
+    <mergeCell ref="G341:G342"/>
+    <mergeCell ref="F339:F340"/>
+    <mergeCell ref="F341:F342"/>
+    <mergeCell ref="F348:F349"/>
+    <mergeCell ref="G348:G349"/>
+    <mergeCell ref="F350:F352"/>
+    <mergeCell ref="G350:G352"/>
+    <mergeCell ref="G353:G354"/>
+    <mergeCell ref="F353:F354"/>
+    <mergeCell ref="F355:F358"/>
+    <mergeCell ref="G355:G358"/>
+    <mergeCell ref="F359:F362"/>
+    <mergeCell ref="G359:G362"/>
+    <mergeCell ref="F363:F365"/>
+    <mergeCell ref="G363:G365"/>
     <mergeCell ref="F374:F376"/>
+    <mergeCell ref="F377:F378"/>
+    <mergeCell ref="F379:F380"/>
+    <mergeCell ref="G377:G378"/>
+    <mergeCell ref="G379:G380"/>
+    <mergeCell ref="F366:F367"/>
+    <mergeCell ref="G366:G367"/>
+    <mergeCell ref="F368:F369"/>
+    <mergeCell ref="G368:G369"/>
+    <mergeCell ref="F370:F373"/>
+    <mergeCell ref="G370:G373"/>
     <mergeCell ref="G374:G376"/>
   </mergeCells>
   <drawing r:id="rId4"/>

</xml_diff>